<commit_message>
perbaiki kolom tabel subsls
</commit_message>
<xml_diff>
--- a/rekap status assignmen 25 juni-2.xlsx
+++ b/rekap status assignmen 25 juni-2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SE2026\monitoring-se2026-ppu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0F28CB3-9C0D-479B-A5E7-4448574BD9EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E4E53C-ABC3-41E6-8D4F-2245945CF766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="query" sheetId="1" r:id="rId1"/>

</xml_diff>